<commit_message>
Add monthly weather update for 2026-5
</commit_message>
<xml_diff>
--- a/workbook/Wind Rain Temp (Active).xlsx
+++ b/workbook/Wind Rain Temp (Active).xlsx
@@ -1854,7 +1854,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -1918,7 +1918,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -2757,7 +2757,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -2821,7 +2821,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -2876,7 +2876,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-CH"/>
         </a:p>
@@ -3715,7 +3715,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -3778,7 +3778,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -4624,7 +4624,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -4688,7 +4688,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5018,7 +5018,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5075,7 +5075,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5404,7 +5404,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5460,7 +5460,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5789,7 +5789,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>
@@ -5846,7 +5846,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="LID4096"/>
           </a:p>

</xml_diff>

<commit_message>
Replace May 2026 weather data with Nordic KNMI area
</commit_message>
<xml_diff>
--- a/workbook/Wind Rain Temp (Active).xlsx
+++ b/workbook/Wind Rain Temp (Active).xlsx
@@ -11196,7 +11196,7 @@
         <v>4.90128</v>
       </c>
       <c r="H65" s="29" t="n">
-        <v>1.67073404788971</v>
+        <v>4.299033641815186</v>
       </c>
       <c r="I65" s="29" t="n"/>
       <c r="J65" s="29" t="n"/>
@@ -14950,7 +14950,7 @@
         <v>1.247521</v>
       </c>
       <c r="H65" s="29" t="n">
-        <v>3.40525661745379</v>
+        <v>2.189102192078867</v>
       </c>
       <c r="I65" s="29" t="n"/>
       <c r="J65" s="29" t="n"/>
@@ -17902,7 +17902,7 @@
         <v>4.437531</v>
       </c>
       <c r="H65" s="29" t="n">
-        <v>12.93547973632815</v>
+        <v>8.457788085937523</v>
       </c>
       <c r="I65" s="29" t="n"/>
       <c r="J65" s="29" t="n"/>

</xml_diff>

<commit_message>
Add monthly weather update for 2026-6
</commit_message>
<xml_diff>
--- a/workbook/Wind Rain Temp (Active).xlsx
+++ b/workbook/Wind Rain Temp (Active).xlsx
@@ -11198,7 +11198,9 @@
       <c r="H65" s="29" t="n">
         <v>4.299033641815186</v>
       </c>
-      <c r="I65" s="29" t="n"/>
+      <c r="I65" s="29" t="n">
+        <v>4.138603687286377</v>
+      </c>
       <c r="J65" s="29" t="n"/>
       <c r="K65" s="29" t="n"/>
       <c r="L65" s="29" t="n"/>
@@ -14952,7 +14954,9 @@
       <c r="H65" s="29" t="n">
         <v>2.189102192078867</v>
       </c>
-      <c r="I65" s="29" t="n"/>
+      <c r="I65" s="29" t="n">
+        <v>3.081081310908</v>
+      </c>
       <c r="J65" s="29" t="n"/>
       <c r="K65" s="29" t="n"/>
       <c r="L65" s="29" t="n"/>
@@ -17904,7 +17908,9 @@
       <c r="H65" s="29" t="n">
         <v>8.457788085937523</v>
       </c>
-      <c r="I65" s="29" t="n"/>
+      <c r="I65" s="29" t="n">
+        <v>13.40517578125002</v>
+      </c>
       <c r="J65" s="29" t="n"/>
       <c r="K65" s="29" t="n"/>
       <c r="L65" s="29" t="n"/>

</xml_diff>